<commit_message>
Final part for python
</commit_message>
<xml_diff>
--- a/data/raw/frapid_base.xlsx
+++ b/data/raw/frapid_base.xlsx
@@ -1,35 +1,80 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10419"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\PID\FRAPID\M2 Ines\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ines/Desktop/MAM2ADMM/VINCENT.INES/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A60D09C-78CE-DD4E-B8B2-DFA8870540EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="2150" windowHeight="0"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="14660" windowHeight="16900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="base de données brute" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>MENIGOZ Charlotte</author>
   </authors>
   <commentList>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>MENIGOZ Charlotte:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>si DLCO réalisable +3</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AH5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -49,247 +94,40 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-si DLCO réalisable +3</t>
+non possible</t>
         </r>
       </text>
     </comment>
-    <comment ref="AH5" authorId="0" shapeId="0">
+    <comment ref="AJ5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>MENIGOZ Charlotte:</t>
         </r>
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-non possible</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AJ5" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>MENIGOZ Charlotte:</t>
+</t>
         </r>
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
-          <t xml:space="preserve">
-non possible sur l'appareil</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BL7" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>MENIGOZ Charlotte:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-essai clinique</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BF17" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>MENIGOZ Charlotte:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-avec SD</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BG18" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>MENIGOZ Charlotte:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-BIP</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BG23" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>MENIGOZ Charlotte:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-DIPNECH + fiborse</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BG27" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>MENIGOZ Charlotte:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-FEPP</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BL28" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>MENIGOZ Charlotte:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-arret à J3</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BG40" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>MENIGOZ Charlotte:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-IPAF</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BG47" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>MENIGOZ Charlotte:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-pneumoconiose</t>
+          <t>non possible sur l'appareil</t>
         </r>
       </text>
     </comment>
@@ -300,60 +138,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="62">
   <si>
-    <t>Patient</t>
-  </si>
-  <si>
-    <t>date_visite</t>
-  </si>
-  <si>
-    <t>naissance</t>
-  </si>
-  <si>
-    <t>sexe</t>
-  </si>
-  <si>
-    <t>poids</t>
-  </si>
-  <si>
-    <t>taille</t>
-  </si>
-  <si>
-    <t>tabac</t>
-  </si>
-  <si>
-    <t>Tabac_PA</t>
-  </si>
-  <si>
-    <t>ATCDfamilial</t>
-  </si>
-  <si>
-    <t>BPCO</t>
-  </si>
-  <si>
-    <t>Resection</t>
-  </si>
-  <si>
-    <t>HTP</t>
-  </si>
-  <si>
-    <t>IMC</t>
-  </si>
-  <si>
-    <t>M0_dyspnée</t>
-  </si>
-  <si>
-    <t>M0_OLD</t>
-  </si>
-  <si>
-    <t>M0_O2déamb</t>
-  </si>
-  <si>
-    <t>M0_CVF(L)</t>
-  </si>
-  <si>
-    <t>M0_CVF(%)</t>
-  </si>
-  <si>
     <t>M0_DLCO(%)</t>
   </si>
   <si>
@@ -363,28 +147,7 @@
     <t>ILD_GAP</t>
   </si>
   <si>
-    <t>index charlson</t>
-  </si>
-  <si>
-    <t>SARC-F</t>
-  </si>
-  <si>
-    <t>Mollet(cm)</t>
-  </si>
-  <si>
     <t>Ishii</t>
-  </si>
-  <si>
-    <t>SARC-Calf</t>
-  </si>
-  <si>
-    <t>Test4m</t>
-  </si>
-  <si>
-    <t>Test5levers</t>
-  </si>
-  <si>
-    <t>handgrip</t>
   </si>
   <si>
     <t>Fried</t>
@@ -417,34 +180,7 @@
     <t>NF</t>
   </si>
   <si>
-    <t>M0_dateEFR</t>
-  </si>
-  <si>
-    <t>masse_maigre</t>
-  </si>
-  <si>
-    <t>masse_muscu</t>
-  </si>
-  <si>
-    <t>masse_grasse</t>
-  </si>
-  <si>
-    <t>Cortico</t>
-  </si>
-  <si>
-    <t>Cancer</t>
-  </si>
-  <si>
     <t>.</t>
-  </si>
-  <si>
-    <t>index_muscu(m2)</t>
-  </si>
-  <si>
-    <t>sarcopénie</t>
-  </si>
-  <si>
-    <t>résistance</t>
   </si>
   <si>
     <t>ASM(0,52)</t>
@@ -453,44 +189,146 @@
     <t>ASM_R</t>
   </si>
   <si>
-    <t>fragile</t>
+    <t>visit_date</t>
   </si>
   <si>
-    <t>pré fragile</t>
+    <t>gender</t>
   </si>
   <si>
-    <t>fragilité</t>
+    <t>weight</t>
   </si>
   <si>
-    <t>Ishii patho</t>
+    <t>height</t>
   </si>
   <si>
-    <t>SARC Calf patho</t>
+    <t>BMI</t>
   </si>
   <si>
-    <t>SARC-F patho</t>
+    <t>smoking</t>
   </si>
   <si>
-    <t>FRAIL patho</t>
+    <t>pack_per_year</t>
   </si>
   <si>
-    <t>EFC patho</t>
+    <t>family_history</t>
   </si>
   <si>
-    <t>GFST path</t>
+    <t>COPD</t>
   </si>
   <si>
-    <t>HAD patho</t>
+    <t>PH</t>
   </si>
   <si>
-    <t>sarcopénie sévère</t>
+    <t>resection</t>
+  </si>
+  <si>
+    <t>cortico</t>
+  </si>
+  <si>
+    <t>cancer</t>
+  </si>
+  <si>
+    <t>M0_dyspnea</t>
+  </si>
+  <si>
+    <t>M0_LTOT</t>
+  </si>
+  <si>
+    <t>M0_walkingO2</t>
+  </si>
+  <si>
+    <t>M0_PFT_date</t>
+  </si>
+  <si>
+    <t>M0_FVCL)</t>
+  </si>
+  <si>
+    <t>M0_FVC(%)</t>
+  </si>
+  <si>
+    <t>charlson_index</t>
+  </si>
+  <si>
+    <t>calf(cm)</t>
+  </si>
+  <si>
+    <t>SARC_F</t>
+  </si>
+  <si>
+    <t>SARC_F_patho</t>
+  </si>
+  <si>
+    <t>SARC_Calf</t>
+  </si>
+  <si>
+    <t>SARC_Calf_patho</t>
+  </si>
+  <si>
+    <t>Ishii_patho</t>
+  </si>
+  <si>
+    <t>walk_time_4m</t>
+  </si>
+  <si>
+    <t>time_5_raise_chair</t>
+  </si>
+  <si>
+    <t>body_fat</t>
+  </si>
+  <si>
+    <t>lean_body_mass</t>
+  </si>
+  <si>
+    <t>muscle_mass</t>
+  </si>
+  <si>
+    <t>resistance</t>
+  </si>
+  <si>
+    <t>muscle_index(m2)</t>
+  </si>
+  <si>
+    <t>sarcopenia</t>
+  </si>
+  <si>
+    <t>severe_sarcopenia</t>
+  </si>
+  <si>
+    <t>frail</t>
+  </si>
+  <si>
+    <t>pre_frail</t>
+  </si>
+  <si>
+    <t>frailty</t>
+  </si>
+  <si>
+    <t>FRAIL_patho</t>
+  </si>
+  <si>
+    <t>EFC_patho</t>
+  </si>
+  <si>
+    <t>GFST_patho</t>
+  </si>
+  <si>
+    <t>HAD_patho</t>
+  </si>
+  <si>
+    <t>birth_year</t>
+  </si>
+  <si>
+    <t>handgrip_strength</t>
+  </si>
+  <si>
+    <t>patient_id</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -512,17 +350,22 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
-      <color indexed="81"/>
+      <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
-      <color indexed="81"/>
+      <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri (Corps)"/>
     </font>
   </fonts>
   <fills count="2">
@@ -594,7 +437,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -611,45 +454,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -929,275 +755,273 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:CE48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.90625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="3.7265625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="4.54296875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="5.36328125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="4.81640625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="5.26953125" style="4" customWidth="1"/>
-    <col min="9" max="9" width="5.36328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="8.90625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="11.453125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="5.36328125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="4.08984375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="6.7265625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="6.54296875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="3.6640625" style="1" customWidth="1"/>
+    <col min="5" max="6" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.33203125" style="4" customWidth="1"/>
+    <col min="9" max="9" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.83203125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="4.1640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="6.6640625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="6.5" style="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5" style="1" customWidth="1"/>
     <col min="18" max="18" width="8" style="1" customWidth="1"/>
-    <col min="19" max="19" width="12.7265625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="11.26953125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="9.7265625" style="1" customWidth="1"/>
-    <col min="22" max="22" width="10.36328125" style="1" customWidth="1"/>
-    <col min="23" max="23" width="11.81640625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="7.90625" style="1" customWidth="1"/>
-    <col min="25" max="25" width="12.90625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="6.6328125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="12.6640625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.33203125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="9.6640625" style="1" customWidth="1"/>
+    <col min="22" max="22" width="10.33203125" style="1" customWidth="1"/>
+    <col min="23" max="23" width="11.83203125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="7.83203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.6640625" style="1" customWidth="1"/>
     <col min="27" max="27" width="12" style="1" customWidth="1"/>
-    <col min="28" max="28" width="9.90625" style="1" customWidth="1"/>
-    <col min="29" max="29" width="8.90625" style="1" customWidth="1"/>
-    <col min="30" max="30" width="14.08984375" style="1" customWidth="1"/>
-    <col min="31" max="31" width="6.81640625" style="1" customWidth="1"/>
-    <col min="32" max="32" width="9.54296875" style="1" customWidth="1"/>
-    <col min="33" max="33" width="6.90625" style="1" customWidth="1"/>
-    <col min="34" max="34" width="10.1796875" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.26953125" style="1" customWidth="1"/>
-    <col min="36" max="36" width="12.36328125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="12.81640625" style="1" customWidth="1"/>
-    <col min="38" max="38" width="12.54296875" style="1" customWidth="1"/>
-    <col min="39" max="39" width="9.1796875" style="1" customWidth="1"/>
-    <col min="40" max="40" width="6.7265625" style="4" customWidth="1"/>
-    <col min="41" max="41" width="9.36328125" style="1" customWidth="1"/>
-    <col min="42" max="42" width="15.7265625" style="4" customWidth="1"/>
-    <col min="43" max="43" width="9.90625" style="8" customWidth="1"/>
-    <col min="44" max="44" width="15.90625" style="8" customWidth="1"/>
+    <col min="28" max="28" width="9.83203125" style="1" customWidth="1"/>
+    <col min="29" max="29" width="8.83203125" style="1" customWidth="1"/>
+    <col min="30" max="30" width="14.1640625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="6.83203125" style="1" customWidth="1"/>
+    <col min="32" max="32" width="9.5" style="1" customWidth="1"/>
+    <col min="33" max="33" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.1640625" style="1" customWidth="1"/>
+    <col min="35" max="35" width="15.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.33203125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="13.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.5" style="1" customWidth="1"/>
+    <col min="39" max="39" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="6.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="15.6640625" style="4" customWidth="1"/>
+    <col min="43" max="43" width="9.83203125" style="6" customWidth="1"/>
+    <col min="44" max="44" width="15.83203125" style="6" customWidth="1"/>
     <col min="45" max="45" width="5" style="1" customWidth="1"/>
     <col min="46" max="46" width="6" style="1" customWidth="1"/>
-    <col min="47" max="47" width="9.26953125" style="1" customWidth="1"/>
-    <col min="48" max="48" width="8.81640625" style="1" customWidth="1"/>
-    <col min="49" max="49" width="5.36328125" style="1" customWidth="1"/>
-    <col min="50" max="50" width="10.7265625" style="1" customWidth="1"/>
-    <col min="51" max="51" width="3.81640625" style="1" customWidth="1"/>
-    <col min="52" max="52" width="9.1796875" style="1" customWidth="1"/>
-    <col min="53" max="53" width="4.90625" style="1" customWidth="1"/>
-    <col min="54" max="54" width="9.1796875" style="1" customWidth="1"/>
-    <col min="55" max="55" width="4.54296875" style="1" customWidth="1"/>
-    <col min="56" max="56" width="9.90625" style="1" customWidth="1"/>
-    <col min="57" max="57" width="5.36328125" style="1" customWidth="1"/>
-    <col min="58" max="58" width="10.453125" style="11" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="10.81640625" style="12" customWidth="1"/>
-    <col min="60" max="60" width="10.36328125" style="12" customWidth="1"/>
-    <col min="61" max="61" width="8.1796875" style="12" customWidth="1"/>
-    <col min="62" max="62" width="11.7265625" style="12" customWidth="1"/>
-    <col min="63" max="63" width="7.54296875" style="12" customWidth="1"/>
-    <col min="64" max="64" width="7" style="12" customWidth="1"/>
-    <col min="65" max="65" width="11.1796875" style="14" customWidth="1"/>
-    <col min="66" max="66" width="11" style="13" customWidth="1"/>
-    <col min="67" max="67" width="11" style="12" customWidth="1"/>
-    <col min="68" max="69" width="10.90625" style="9"/>
-    <col min="70" max="70" width="11.54296875" style="1" customWidth="1"/>
-    <col min="71" max="71" width="10.90625" style="10"/>
+    <col min="47" max="47" width="9.33203125" style="1" customWidth="1"/>
+    <col min="48" max="48" width="8.83203125" style="1" customWidth="1"/>
+    <col min="49" max="49" width="5.33203125" style="1" customWidth="1"/>
+    <col min="50" max="50" width="10.6640625" style="1" customWidth="1"/>
+    <col min="51" max="51" width="3.83203125" style="1" customWidth="1"/>
+    <col min="52" max="52" width="9.1640625" style="1" customWidth="1"/>
+    <col min="53" max="53" width="4.83203125" style="1" customWidth="1"/>
+    <col min="54" max="54" width="9.1640625" style="1" customWidth="1"/>
+    <col min="55" max="55" width="4.5" style="1" customWidth="1"/>
+    <col min="56" max="56" width="9.83203125" style="1" customWidth="1"/>
+    <col min="57" max="57" width="5.33203125" style="1" customWidth="1"/>
+    <col min="58" max="58" width="10.5" style="7" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="10.83203125" style="1" customWidth="1"/>
+    <col min="60" max="60" width="10.33203125" style="1" customWidth="1"/>
+    <col min="61" max="61" width="8.1640625" style="1" customWidth="1"/>
+    <col min="62" max="62" width="11.6640625" style="1" customWidth="1"/>
+    <col min="63" max="63" width="7.5" style="1" customWidth="1"/>
+    <col min="64" max="64" width="7" style="1" customWidth="1"/>
+    <col min="65" max="65" width="11.1640625" style="3" customWidth="1"/>
+    <col min="66" max="66" width="11" style="8" customWidth="1"/>
+    <col min="67" max="67" width="11" style="1" customWidth="1"/>
+    <col min="68" max="69" width="10.83203125" style="1"/>
+    <col min="70" max="70" width="11.5" style="1" customWidth="1"/>
+    <col min="71" max="71" width="10.83203125" style="6"/>
     <col min="72" max="72" width="8" style="1" customWidth="1"/>
-    <col min="73" max="73" width="12.7265625" style="1" customWidth="1"/>
-    <col min="74" max="74" width="11.26953125" style="1" customWidth="1"/>
-    <col min="75" max="75" width="9.7265625" style="1" customWidth="1"/>
-    <col min="76" max="77" width="10.36328125" style="1" customWidth="1"/>
+    <col min="73" max="73" width="12.6640625" style="1" customWidth="1"/>
+    <col min="74" max="74" width="11.33203125" style="1" customWidth="1"/>
+    <col min="75" max="75" width="9.6640625" style="1" customWidth="1"/>
+    <col min="76" max="77" width="10.33203125" style="1" customWidth="1"/>
     <col min="78" max="78" width="14" style="2" customWidth="1"/>
-    <col min="79" max="79" width="16.7265625" style="1" customWidth="1"/>
-    <col min="80" max="80" width="10.90625" style="1"/>
-    <col min="81" max="81" width="16.36328125" style="1" customWidth="1"/>
-    <col min="82" max="16384" width="10.90625" style="1"/>
+    <col min="79" max="79" width="16.6640625" style="1" customWidth="1"/>
+    <col min="80" max="80" width="10.83203125" style="1"/>
+    <col min="81" max="81" width="16.33203125" style="1" customWidth="1"/>
+    <col min="82" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="X1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AG1" t="s">
         <v>43</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="AH1" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="Q1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="AI1" s="1" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="AM1" s="1" t="s">
         <v>48</v>
       </c>
       <c r="AN1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="AP1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AQ1" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="AO1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AP1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="AQ1" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="AR1" s="8" t="s">
-        <v>61</v>
+      <c r="AR1" s="6" t="s">
+        <v>51</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="AX1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="BB1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="AY1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="BD1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="BA1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="BB1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="BC1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="BD1" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="BE1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="BF1" s="15"/>
-      <c r="BG1" s="16"/>
-      <c r="BH1" s="16"/>
-      <c r="BI1" s="16"/>
-      <c r="BJ1" s="16"/>
-      <c r="BK1" s="16"/>
-      <c r="BL1" s="16"/>
-      <c r="BM1" s="17"/>
-      <c r="BN1" s="18"/>
+        <v>9</v>
+      </c>
+      <c r="BF1" s="9"/>
+      <c r="BG1" s="10"/>
+      <c r="BH1" s="10"/>
+      <c r="BI1" s="10"/>
+      <c r="BJ1" s="10"/>
+      <c r="BK1" s="10"/>
+      <c r="BL1" s="10"/>
+      <c r="BM1" s="11"/>
+      <c r="BN1" s="12"/>
     </row>
-    <row r="2" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1212,7 +1036,7 @@
         <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F2" s="1">
         <v>60</v>
@@ -1225,7 +1049,7 @@
         <v>20.761245674740486</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J2" s="1">
         <v>10</v>
@@ -1336,11 +1160,11 @@
         <f>IF(BC2&gt;=11,1,0)</f>
         <v>0</v>
       </c>
-      <c r="BO2" s="14"/>
+      <c r="BO2" s="3"/>
       <c r="BV2" s="3"/>
       <c r="CA2" s="3"/>
     </row>
-    <row r="3" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1355,7 +1179,7 @@
         <v>72</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F3" s="1">
         <v>95</v>
@@ -1368,7 +1192,7 @@
         <v>37.109375</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K3" s="1">
         <v>0</v>
@@ -1397,16 +1221,16 @@
       <c r="S3" s="1">
         <v>0</v>
       </c>
-      <c r="T3" s="6">
+      <c r="T3" s="3">
         <v>45188</v>
       </c>
-      <c r="U3" s="7">
+      <c r="U3" s="1">
         <v>2.12</v>
       </c>
-      <c r="V3" s="7">
+      <c r="V3" s="1">
         <v>88</v>
       </c>
-      <c r="W3" s="7">
+      <c r="W3" s="1">
         <v>30</v>
       </c>
       <c r="X3" s="5">
@@ -1475,11 +1299,11 @@
         <f>AN3/G3/G3</f>
         <v>3.9980670306691448</v>
       </c>
-      <c r="AQ3" s="8">
+      <c r="AQ3" s="6">
         <f>IF(AND(E3="F",OR(AI3&lt;16,AH3&gt;15),AP3&lt;5.5),1,IF(AND(E3="M",OR(AI3&lt;27,AH3&gt;15),AP3&lt;7),1,0))</f>
         <v>0</v>
       </c>
-      <c r="AR3" s="8">
+      <c r="AR3" s="6">
         <f>IF(AND(AQ3=1,AG3&gt;4),1,0)</f>
         <v>0</v>
       </c>
@@ -1529,13 +1353,10 @@
       <c r="BE3" s="1">
         <v>39</v>
       </c>
-      <c r="BO3" s="14"/>
-      <c r="BV3" s="6"/>
-      <c r="BW3" s="7"/>
-      <c r="BX3" s="7"/>
-      <c r="BY3" s="7"/>
+      <c r="BO3" s="3"/>
+      <c r="BV3" s="3"/>
     </row>
-    <row r="4" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1550,7 +1371,7 @@
         <v>83</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F4" s="1">
         <v>54</v>
@@ -1563,7 +1384,7 @@
         <v>21.631148854350261</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J4" s="1">
         <v>35</v>
@@ -1673,11 +1494,11 @@
         <f>AN4/G4/G4</f>
         <v>3.8647209238446223</v>
       </c>
-      <c r="AQ4" s="8">
+      <c r="AQ4" s="6">
         <f>IF(AND(E4="F",OR(AI4&lt;16,AH4&gt;15),AP4&lt;5.5),1,IF(AND(E4="M",OR(AI4&lt;27,AH4&gt;15),AP4&lt;7),1,0))</f>
         <v>1</v>
       </c>
-      <c r="AR4" s="8">
+      <c r="AR4" s="6">
         <f t="shared" ref="AR4:AR32" si="15">IF(AND(AQ4=1,AG4&gt;4),1,0)</f>
         <v>0</v>
       </c>
@@ -1728,10 +1549,10 @@
         <f>7*15</f>
         <v>105</v>
       </c>
-      <c r="BO4" s="14"/>
+      <c r="BO4" s="3"/>
       <c r="BV4" s="3"/>
     </row>
-    <row r="5" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1746,7 +1567,7 @@
         <v>76</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F5" s="1">
         <v>175</v>
@@ -1759,7 +1580,7 @@
         <v>60.553633217993081</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J5" s="1">
         <v>40</v>
@@ -1888,10 +1709,10 @@
       <c r="BE5" s="1">
         <v>77</v>
       </c>
-      <c r="BO5" s="14"/>
+      <c r="BO5" s="3"/>
       <c r="BV5" s="3"/>
     </row>
-    <row r="6" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1906,7 +1727,7 @@
         <v>77</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F6" s="1">
         <v>77</v>
@@ -1919,7 +1740,7 @@
         <v>27.281746031746035</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J6" s="1">
         <v>60</v>
@@ -2018,11 +1839,11 @@
         <f t="shared" ref="AO6:AO16" si="17">0.52*AL6</f>
         <v>28.6</v>
       </c>
-      <c r="AQ6" s="8">
+      <c r="AQ6" s="6">
         <f t="shared" ref="AQ6:AQ16" si="18">IF(AND(E6="F",OR(AI6&lt;16,AH6&gt;15),AP6&lt;5.5),1,IF(AND(E6="M",OR(AI6&lt;27,AH6&gt;15),AP6&lt;7),1,0))</f>
         <v>1</v>
       </c>
-      <c r="AR6" s="8">
+      <c r="AR6" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -2074,7 +1895,7 @@
       </c>
       <c r="BV6" s="3"/>
     </row>
-    <row r="7" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2089,7 +1910,7 @@
         <v>79</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F7" s="1">
         <v>90</v>
@@ -2102,7 +1923,7 @@
         <v>29.0547520661157</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J7" s="1">
         <v>40</v>
@@ -2212,11 +2033,11 @@
         <f t="shared" ref="AP7:AP16" si="20">AN7/G7/G7</f>
         <v>5.1951866277611813</v>
       </c>
-      <c r="AQ7" s="8">
+      <c r="AQ7" s="6">
         <f t="shared" si="18"/>
         <v>1</v>
       </c>
-      <c r="AR7" s="8">
+      <c r="AR7" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -2266,10 +2087,10 @@
       <c r="BE7" s="1">
         <v>67</v>
       </c>
-      <c r="BO7" s="14"/>
+      <c r="BO7" s="3"/>
       <c r="BV7" s="3"/>
     </row>
-    <row r="8" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2284,7 +2105,7 @@
         <v>70</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F8" s="1">
         <v>88</v>
@@ -2297,7 +2118,7 @@
         <v>28.73469387755102</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J8" s="1">
         <v>35</v>
@@ -2407,11 +2228,11 @@
         <f t="shared" si="20"/>
         <v>5.1377400431538254</v>
       </c>
-      <c r="AQ8" s="8">
+      <c r="AQ8" s="6">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="AR8" s="8">
+      <c r="AR8" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -2461,10 +2282,10 @@
       <c r="BE8" s="1">
         <v>58</v>
       </c>
-      <c r="BO8" s="14"/>
+      <c r="BO8" s="3"/>
       <c r="BV8" s="3"/>
     </row>
-    <row r="9" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2479,7 +2300,7 @@
         <v>76</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F9" s="1">
         <v>84</v>
@@ -2492,7 +2313,7 @@
         <v>28.393726338561386</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J9" s="1">
         <v>10</v>
@@ -2602,11 +2423,11 @@
         <f t="shared" si="20"/>
         <v>5.0765095894791141</v>
       </c>
-      <c r="AQ9" s="8">
+      <c r="AQ9" s="6">
         <f t="shared" si="18"/>
         <v>1</v>
       </c>
-      <c r="AR9" s="8">
+      <c r="AR9" s="6">
         <f t="shared" si="15"/>
         <v>1</v>
       </c>
@@ -2659,7 +2480,7 @@
       <c r="BV9" s="3"/>
       <c r="CE9" s="3"/>
     </row>
-    <row r="10" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2674,7 +2495,7 @@
         <v>75</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F10" s="1">
         <v>64</v>
@@ -2687,7 +2508,7 @@
         <v>26.298487836949374</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K10" s="1">
         <v>1</v>
@@ -2794,11 +2615,11 @@
         <f t="shared" si="20"/>
         <v>2.7153598980328568</v>
       </c>
-      <c r="AQ10" s="8">
+      <c r="AQ10" s="6">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="AR10" s="8">
+      <c r="AR10" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -2850,7 +2671,7 @@
       </c>
       <c r="BV10" s="3"/>
     </row>
-    <row r="11" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2865,7 +2686,7 @@
         <v>73</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F11" s="1">
         <v>76</v>
@@ -2878,7 +2699,7 @@
         <v>25.689561925365062</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J11" s="1">
         <v>60</v>
@@ -2988,11 +2809,11 @@
         <f t="shared" si="20"/>
         <v>4.5923992931689055</v>
       </c>
-      <c r="AQ11" s="8">
+      <c r="AQ11" s="6">
         <f t="shared" si="18"/>
         <v>1</v>
       </c>
-      <c r="AR11" s="8">
+      <c r="AR11" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -3042,10 +2863,10 @@
       <c r="BE11" s="1">
         <v>70</v>
       </c>
-      <c r="BO11" s="14"/>
+      <c r="BO11" s="3"/>
       <c r="BV11" s="3"/>
     </row>
-    <row r="12" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -3060,7 +2881,7 @@
         <v>80</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F12" s="1">
         <v>50</v>
@@ -3073,7 +2894,7 @@
         <v>17.301038062283737</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K12" s="1">
         <v>0</v>
@@ -3180,11 +3001,11 @@
         <f t="shared" si="20"/>
         <v>1.7198200484013009</v>
       </c>
-      <c r="AQ12" s="8">
+      <c r="AQ12" s="6">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="AR12" s="8">
+      <c r="AR12" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -3237,7 +3058,7 @@
       </c>
       <c r="BV12" s="3"/>
     </row>
-    <row r="13" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -3252,7 +3073,7 @@
         <v>66</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F13" s="1">
         <v>96</v>
@@ -3265,7 +3086,7 @@
         <v>34.013605442176875</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="J13" s="1">
         <v>40</v>
@@ -3372,11 +3193,11 @@
         <f t="shared" si="20"/>
         <v>6.0821805123179224</v>
       </c>
-      <c r="AQ13" s="8">
+      <c r="AQ13" s="6">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="AR13" s="8">
+      <c r="AR13" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -3428,7 +3249,7 @@
       </c>
       <c r="BV13" s="3"/>
     </row>
-    <row r="14" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -3443,7 +3264,7 @@
         <v>88</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F14" s="1">
         <v>65</v>
@@ -3456,7 +3277,7 @@
         <v>25.076193048107708</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J14" s="1">
         <v>10</v>
@@ -3566,11 +3387,11 @@
         <f t="shared" si="20"/>
         <v>4.4818085914895249</v>
       </c>
-      <c r="AQ14" s="8">
+      <c r="AQ14" s="6">
         <f t="shared" si="18"/>
         <v>1</v>
       </c>
-      <c r="AR14" s="8">
+      <c r="AR14" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -3623,7 +3444,7 @@
       </c>
       <c r="BV14" s="3"/>
     </row>
-    <row r="15" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -3638,7 +3459,7 @@
         <v>78</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F15" s="1">
         <v>80</v>
@@ -3651,7 +3472,7 @@
         <v>25.535446391522232</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J15" s="1">
         <v>40</v>
@@ -3761,11 +3582,11 @@
         <f t="shared" si="20"/>
         <v>4.5653141109032456</v>
       </c>
-      <c r="AQ15" s="8">
+      <c r="AQ15" s="6">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="AR15" s="8">
+      <c r="AR15" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -3818,7 +3639,7 @@
       </c>
       <c r="BV15" s="3"/>
     </row>
-    <row r="16" spans="1:83" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:83" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -3833,7 +3654,7 @@
         <v>71</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F16" s="1">
         <v>37</v>
@@ -3846,7 +3667,7 @@
         <v>16.444444444444446</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K16" s="1">
         <v>1</v>
@@ -3953,11 +3774,11 @@
         <f t="shared" si="20"/>
         <v>1.5327733134920638</v>
       </c>
-      <c r="AQ16" s="8">
+      <c r="AQ16" s="6">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="AR16" s="8">
+      <c r="AR16" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -4009,7 +3830,7 @@
       </c>
       <c r="BV16" s="3"/>
     </row>
-    <row r="17" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -4024,7 +3845,7 @@
         <v>82</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F17" s="1">
         <v>80</v>
@@ -4037,7 +3858,7 @@
         <v>26.729927495071671</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K17" s="1">
         <v>0</v>
@@ -4120,10 +3941,6 @@
       <c r="AI17" s="1">
         <v>22</v>
       </c>
-      <c r="AJ17" s="7"/>
-      <c r="AK17" s="7"/>
-      <c r="AL17" s="7"/>
-      <c r="AM17" s="7"/>
       <c r="AS17" s="1">
         <v>1</v>
       </c>
@@ -4173,7 +3990,7 @@
       </c>
       <c r="BV17" s="3"/>
     </row>
-    <row r="18" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -4188,7 +4005,7 @@
         <v>70</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F18" s="1">
         <v>64</v>
@@ -4201,7 +4018,7 @@
         <v>20.1994697639187</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J18" s="1">
         <v>5</v>
@@ -4218,13 +4035,13 @@
       <c r="N18" s="1">
         <v>0</v>
       </c>
-      <c r="O18" s="7">
-        <v>0</v>
-      </c>
-      <c r="P18" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="7">
+      <c r="O18" s="1">
+        <v>0</v>
+      </c>
+      <c r="P18" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
@@ -4243,7 +4060,7 @@
         <v>99</v>
       </c>
       <c r="W18" s="1" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="X18" s="5">
         <f>IF(E18="M",1,0)+IF(D18&lt;61,0,IF(D18&lt;=65,1,2))+IF(V18&gt;=75,0,IF(V18&gt;=50,1,2))+IF(W18&gt;=55,0,IF(W18&gt;=36,1,2))+IF(OR(BG20="FPI",BG20="inclassable"),0,-2)</f>
@@ -4311,11 +4128,11 @@
         <f t="shared" ref="AP18:AP32" si="23">AN18/G18/G18</f>
         <v>3.6100976982185244</v>
       </c>
-      <c r="AQ18" s="8">
+      <c r="AQ18" s="6">
         <f t="shared" ref="AQ18:AQ32" si="24">IF(AND(E18="F",OR(AI18&lt;16,AH18&gt;15),AP18&lt;5.5),1,IF(AND(E18="M",OR(AI18&lt;27,AH18&gt;15),AP18&lt;7),1,0))</f>
         <v>0</v>
       </c>
-      <c r="AR18" s="8">
+      <c r="AR18" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -4366,10 +4183,9 @@
         <f>5+7+3+7+3+4+7+4+7+6+7+4+7+5+7</f>
         <v>83</v>
       </c>
-      <c r="BR18" s="7"/>
       <c r="BV18" s="3"/>
     </row>
-    <row r="19" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -4384,7 +4200,7 @@
         <v>83</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F19" s="1">
         <v>89</v>
@@ -4397,7 +4213,7 @@
         <v>30.79584775086505</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J19" s="1">
         <v>35</v>
@@ -4507,11 +4323,11 @@
         <f t="shared" si="23"/>
         <v>5.506425052665695</v>
       </c>
-      <c r="AQ19" s="8">
+      <c r="AQ19" s="6">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="AR19" s="8">
+      <c r="AR19" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -4564,7 +4380,7 @@
       </c>
       <c r="BV19" s="3"/>
     </row>
-    <row r="20" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -4579,7 +4395,7 @@
         <v>71</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F20" s="1">
         <v>87</v>
@@ -4592,7 +4408,7 @@
         <v>28.735632183908045</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="K20" s="1">
         <v>0</v>
@@ -4699,11 +4515,11 @@
         <f t="shared" si="23"/>
         <v>5.1379364384250259</v>
       </c>
-      <c r="AQ20" s="8">
+      <c r="AQ20" s="6">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="AR20" s="8">
+      <c r="AR20" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -4756,7 +4572,7 @@
       </c>
       <c r="BV20" s="3"/>
     </row>
-    <row r="21" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -4771,7 +4587,7 @@
         <v>80</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F21" s="1">
         <v>53</v>
@@ -4784,7 +4600,7 @@
         <v>18.125235115078144</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K21" s="1">
         <v>0</v>
@@ -4891,11 +4707,11 @@
         <f t="shared" si="23"/>
         <v>3.238355200510981</v>
       </c>
-      <c r="AQ21" s="8">
+      <c r="AQ21" s="6">
         <f t="shared" si="24"/>
         <v>1</v>
       </c>
-      <c r="AR21" s="8">
+      <c r="AR21" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -4948,7 +4764,7 @@
       </c>
       <c r="BV21" s="3"/>
     </row>
-    <row r="22" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -4963,7 +4779,7 @@
         <v>79</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F22" s="1">
         <v>70</v>
@@ -4976,7 +4792,7 @@
         <v>24.221453287197235</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K22" s="1">
         <v>0</v>
@@ -5083,11 +4899,11 @@
         <f t="shared" si="23"/>
         <v>4.3294831168259922</v>
       </c>
-      <c r="AQ22" s="8">
+      <c r="AQ22" s="6">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="AR22" s="8">
+      <c r="AR22" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -5140,7 +4956,7 @@
       </c>
       <c r="BV22" s="3"/>
     </row>
-    <row r="23" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -5155,7 +4971,7 @@
         <v>75</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F23" s="1">
         <v>109</v>
@@ -5168,7 +4984,7 @@
         <v>30.193905817174517</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J23" s="1">
         <v>30</v>
@@ -5275,11 +5091,11 @@
         <f t="shared" si="23"/>
         <v>5.3997946559458736</v>
       </c>
-      <c r="AQ23" s="8">
+      <c r="AQ23" s="6">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="AR23" s="8">
+      <c r="AR23" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -5332,7 +5148,7 @@
       </c>
       <c r="BV23" s="3"/>
     </row>
-    <row r="24" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -5347,7 +5163,7 @@
         <v>79</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F24" s="1">
         <v>94</v>
@@ -5360,7 +5176,7 @@
         <v>36.71875</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J24" s="1">
         <v>22</v>
@@ -5402,7 +5218,7 @@
         <v>79</v>
       </c>
       <c r="W24" s="1" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="X24" s="5">
         <f t="shared" si="25"/>
@@ -5470,11 +5286,11 @@
         <f t="shared" si="23"/>
         <v>6.5657541639182053</v>
       </c>
-      <c r="AQ24" s="8">
+      <c r="AQ24" s="6">
         <f t="shared" si="24"/>
         <v>1</v>
       </c>
-      <c r="AR24" s="8">
+      <c r="AR24" s="6">
         <f t="shared" si="15"/>
         <v>1</v>
       </c>
@@ -5527,7 +5343,7 @@
       </c>
       <c r="BV24" s="3"/>
     </row>
-    <row r="25" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -5542,7 +5358,7 @@
         <v>80</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F25" s="1">
         <v>92</v>
@@ -5555,7 +5371,7 @@
         <v>28.082170873904946</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J25" s="1">
         <v>25</v>
@@ -5665,11 +5481,11 @@
         <f t="shared" si="23"/>
         <v>5.0212800057783094</v>
       </c>
-      <c r="AQ25" s="8">
+      <c r="AQ25" s="6">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="AR25" s="8">
+      <c r="AR25" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -5712,10 +5528,9 @@
       <c r="BE25" s="1">
         <v>70</v>
       </c>
-      <c r="BP25" s="1"/>
       <c r="BV25" s="3"/>
     </row>
-    <row r="26" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -5730,7 +5545,7 @@
         <v>67</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F26" s="1">
         <v>64.5</v>
@@ -5743,7 +5558,7 @@
         <v>23.406880534184936</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J26" s="1">
         <v>49</v>
@@ -5853,11 +5668,11 @@
         <f t="shared" si="23"/>
         <v>4.1833096715998712</v>
       </c>
-      <c r="AQ26" s="8">
+      <c r="AQ26" s="6">
         <f t="shared" si="24"/>
         <v>1</v>
       </c>
-      <c r="AR26" s="8">
+      <c r="AR26" s="6">
         <f t="shared" si="15"/>
         <v>1</v>
       </c>
@@ -5909,7 +5724,7 @@
       </c>
       <c r="BV26" s="3"/>
     </row>
-    <row r="27" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -5924,7 +5739,7 @@
         <v>69</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F27" s="1">
         <v>55</v>
@@ -5937,7 +5752,7 @@
         <v>24.121749046094472</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K27" s="1">
         <v>0</v>
@@ -6044,11 +5859,11 @@
         <f t="shared" si="23"/>
         <v>2.4362650745585372</v>
       </c>
-      <c r="AQ27" s="8">
+      <c r="AQ27" s="6">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="AR27" s="8">
+      <c r="AR27" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -6100,7 +5915,7 @@
       </c>
       <c r="BV27" s="3"/>
     </row>
-    <row r="28" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -6115,7 +5930,7 @@
         <v>70</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F28" s="1">
         <v>70</v>
@@ -6128,7 +5943,7 @@
         <v>26.026174895895306</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J28" s="1">
         <v>12</v>
@@ -6232,11 +6047,11 @@
         <f t="shared" si="23"/>
         <v>2.7178991044871252</v>
       </c>
-      <c r="AQ28" s="8">
+      <c r="AQ28" s="6">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="AR28" s="8">
+      <c r="AR28" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -6287,7 +6102,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -6302,7 +6117,7 @@
         <v>73</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F29" s="1">
         <v>85</v>
@@ -6315,7 +6130,7 @@
         <v>29.760862714890933</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J29" s="1">
         <v>30</v>
@@ -6457,7 +6272,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -6472,7 +6287,7 @@
         <v>75</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F30" s="1">
         <v>82</v>
@@ -6485,7 +6300,7 @@
         <v>26.173832551310287</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K30" s="1">
         <v>1</v>
@@ -6592,11 +6407,11 @@
         <f t="shared" si="23"/>
         <v>4.6795011298560532</v>
       </c>
-      <c r="AQ30" s="8">
+      <c r="AQ30" s="6">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="AR30" s="8">
+      <c r="AR30" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -6647,7 +6462,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="31" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -6662,7 +6477,7 @@
         <v>79</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F31" s="1">
         <v>68</v>
@@ -6675,7 +6490,7 @@
         <v>22.460034350640772</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J31" s="1">
         <v>40</v>
@@ -6782,11 +6597,11 @@
         <f t="shared" si="23"/>
         <v>4.014463764504284</v>
       </c>
-      <c r="AQ31" s="8">
+      <c r="AQ31" s="6">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="AR31" s="8">
+      <c r="AR31" s="6">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -6837,7 +6652,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:74" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -6852,7 +6667,7 @@
         <v>78</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F32" s="1">
         <v>62</v>
@@ -6865,7 +6680,7 @@
         <v>27.555555555555557</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K32" s="1">
         <v>0</v>
@@ -6969,11 +6784,11 @@
         <f t="shared" si="23"/>
         <v>2.8329490106544899</v>
       </c>
-      <c r="AQ32" s="8">
+      <c r="AQ32" s="6">
         <f t="shared" si="24"/>
         <v>1</v>
       </c>
-      <c r="AR32" s="8">
+      <c r="AR32" s="6">
         <f t="shared" si="15"/>
         <v>1</v>
       </c>
@@ -7024,7 +6839,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -7039,7 +6854,7 @@
         <v>81</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F33" s="1">
         <v>93</v>
@@ -7052,7 +6867,7 @@
         <v>28.703703703703702</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J33" s="1">
         <v>20</v>
@@ -7170,7 +6985,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="34" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -7185,7 +7000,7 @@
         <v>84</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F34" s="1">
         <v>50</v>
@@ -7198,7 +7013,7 @@
         <v>19.051973784484069</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J34" s="1">
         <v>1</v>
@@ -7305,11 +7120,11 @@
         <f t="shared" ref="AP34:AP35" si="30">AN34/G34/G34</f>
         <v>1.8937130478771014</v>
       </c>
-      <c r="AQ34" s="8">
+      <c r="AQ34" s="6">
         <f t="shared" ref="AQ34:AQ35" si="31">IF(AND(E34="F",OR(AI34&lt;16,AH34&gt;15),AP34&lt;5.5),1,IF(AND(E34="M",OR(AI34&lt;27,AH34&gt;15),AP34&lt;7),1,0))</f>
         <v>1</v>
       </c>
-      <c r="AR34" s="8">
+      <c r="AR34" s="6">
         <f t="shared" ref="AR34:AR35" si="32">IF(AND(AQ34=1,AG34&gt;4),1,0)</f>
         <v>1</v>
       </c>
@@ -7362,7 +7177,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -7377,7 +7192,7 @@
         <v>69</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F35" s="1">
         <v>97</v>
@@ -7390,7 +7205,7 @@
         <v>32.787993510005407</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J35" s="1">
         <v>40</v>
@@ -7500,11 +7315,11 @@
         <f t="shared" si="30"/>
         <v>5.8630224478096276</v>
       </c>
-      <c r="AQ35" s="8">
+      <c r="AQ35" s="6">
         <f t="shared" si="31"/>
         <v>0</v>
       </c>
-      <c r="AR35" s="8">
+      <c r="AR35" s="6">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
@@ -7557,7 +7372,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -7572,7 +7387,7 @@
         <v>75</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F36" s="1">
         <v>104</v>
@@ -7585,7 +7400,7 @@
         <v>32.098765432098766</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J36" s="1">
         <v>50</v>
@@ -7717,7 +7532,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="37" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -7732,7 +7547,7 @@
         <v>89</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F37" s="1">
         <v>33</v>
@@ -7745,7 +7560,7 @@
         <v>15.27141468832431</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K37" s="1">
         <v>0</v>
@@ -7859,7 +7674,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="38" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -7874,7 +7689,7 @@
         <v>71</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F38" s="1">
         <v>77</v>
@@ -7887,7 +7702,7 @@
         <v>28.282828282828287</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J38" s="1">
         <v>2</v>
@@ -7997,11 +7812,11 @@
         <f t="shared" ref="AP38" si="36">AN38/G38/G38</f>
         <v>5.0561290455117973</v>
       </c>
-      <c r="AQ38" s="8">
+      <c r="AQ38" s="6">
         <f t="shared" ref="AQ38" si="37">IF(AND(E38="F",OR(AI38&lt;16,AH38&gt;15),AP38&lt;5.5),1,IF(AND(E38="M",OR(AI38&lt;27,AH38&gt;15),AP38&lt;7),1,0))</f>
         <v>0</v>
       </c>
-      <c r="AR38" s="8">
+      <c r="AR38" s="6">
         <f t="shared" ref="AR38" si="38">IF(AND(AQ38=1,AG38&gt;4),1,0)</f>
         <v>0</v>
       </c>
@@ -8054,7 +7869,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="39" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -8069,7 +7884,7 @@
         <v>76</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F39" s="1">
         <v>86</v>
@@ -8082,7 +7897,7 @@
         <v>27.763429752066116</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J39" s="1">
         <v>10</v>
@@ -8192,11 +8007,11 @@
         <f t="shared" ref="AP39" si="41">AN39/G39/G39</f>
         <v>4.9639688917807181</v>
       </c>
-      <c r="AQ39" s="8">
+      <c r="AQ39" s="6">
         <f t="shared" ref="AQ39" si="42">IF(AND(E39="F",OR(AI39&lt;16,AH39&gt;15),AP39&lt;5.5),1,IF(AND(E39="M",OR(AI39&lt;27,AH39&gt;15),AP39&lt;7),1,0))</f>
         <v>0</v>
       </c>
-      <c r="AR39" s="8">
+      <c r="AR39" s="6">
         <f t="shared" ref="AR39" si="43">IF(AND(AQ39=1,AG39&gt;4),1,0)</f>
         <v>0</v>
       </c>
@@ -8249,7 +8064,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -8264,7 +8079,7 @@
         <v>69</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F40" s="1">
         <v>57</v>
@@ -8277,7 +8092,7 @@
         <v>20.9366391184573</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J40" s="1">
         <v>8</v>
@@ -8387,11 +8202,11 @@
         <f t="shared" ref="AP40:AP48" si="46">AN40/G40/G40</f>
         <v>3.7410590986056036</v>
       </c>
-      <c r="AQ40" s="8">
+      <c r="AQ40" s="6">
         <f t="shared" ref="AQ40" si="47">IF(AND(E40="F",OR(AI40&lt;16,AH40&gt;15),AP40&lt;5.5),1,IF(AND(E40="M",OR(AI40&lt;27,AH40&gt;15),AP40&lt;7),1,0))</f>
         <v>0</v>
       </c>
-      <c r="AR40" s="8">
+      <c r="AR40" s="6">
         <f t="shared" ref="AR40" si="48">IF(AND(AQ40=1,AG40&gt;4),1,0)</f>
         <v>0</v>
       </c>
@@ -8444,7 +8259,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="41" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -8459,7 +8274,7 @@
         <v>75</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F41" s="1">
         <v>100</v>
@@ -8472,7 +8287,7 @@
         <v>39.555397333966212</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J41" s="1">
         <v>10</v>
@@ -8582,11 +8397,11 @@
         <f t="shared" si="46"/>
         <v>7.0735240150080188</v>
       </c>
-      <c r="AQ41" s="8">
+      <c r="AQ41" s="6">
         <f t="shared" ref="AQ41:AQ48" si="49">IF(AND(E41="F",OR(AI41&lt;16,AH41&gt;15),AP41&lt;5.5),1,IF(AND(E41="M",OR(AI41&lt;27,AH41&gt;15),AP41&lt;7),1,0))</f>
         <v>0</v>
       </c>
-      <c r="AR41" s="8">
+      <c r="AR41" s="6">
         <f t="shared" ref="AR41:AR48" si="50">IF(AND(AQ41=1,AG41&gt;4),1,0)</f>
         <v>0</v>
       </c>
@@ -8639,7 +8454,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="42" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -8654,7 +8469,7 @@
         <v>78</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F42" s="1">
         <v>62</v>
@@ -8667,7 +8482,7 @@
         <v>22.230987127541326</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J42" s="1">
         <v>5</v>
@@ -8777,11 +8592,11 @@
         <f t="shared" si="46"/>
         <v>3.9729426876611775</v>
       </c>
-      <c r="AQ42" s="8">
+      <c r="AQ42" s="6">
         <f t="shared" si="49"/>
         <v>0</v>
       </c>
-      <c r="AR42" s="8">
+      <c r="AR42" s="6">
         <f t="shared" si="50"/>
         <v>0</v>
       </c>
@@ -8833,7 +8648,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -8848,7 +8663,7 @@
         <v>87</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F43" s="1">
         <v>87</v>
@@ -8861,7 +8676,7 @@
         <v>30.461118308182488</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J43" s="1">
         <v>25</v>
@@ -8971,11 +8786,11 @@
         <f t="shared" si="46"/>
         <v>5.446439569756687</v>
       </c>
-      <c r="AQ43" s="8">
+      <c r="AQ43" s="6">
         <f t="shared" si="49"/>
         <v>1</v>
       </c>
-      <c r="AR43" s="8">
+      <c r="AR43" s="6">
         <f t="shared" si="50"/>
         <v>1</v>
       </c>
@@ -9012,7 +8827,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -9027,7 +8842,7 @@
         <v>84</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F44" s="1">
         <v>37</v>
@@ -9040,7 +8855,7 @@
         <v>18.349533822654237</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="K44" s="1">
         <v>0</v>
@@ -9138,11 +8953,11 @@
         <f t="shared" si="46"/>
         <v>1.7103017514071295</v>
       </c>
-      <c r="AQ44" s="8">
+      <c r="AQ44" s="6">
         <f t="shared" si="49"/>
         <v>1</v>
       </c>
-      <c r="AR44" s="8">
+      <c r="AR44" s="6">
         <f t="shared" si="50"/>
         <v>1</v>
       </c>
@@ -9193,7 +9008,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="45" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -9208,7 +9023,7 @@
         <v>79</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F45" s="1">
         <v>71</v>
@@ -9221,7 +9036,7 @@
         <v>23.722810651876109</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J45" s="1">
         <v>10</v>
@@ -9331,11 +9146,11 @@
         <f t="shared" si="46"/>
         <v>4.2404814609238839</v>
       </c>
-      <c r="AQ45" s="8">
+      <c r="AQ45" s="6">
         <f t="shared" si="49"/>
         <v>0</v>
       </c>
-      <c r="AR45" s="8">
+      <c r="AR45" s="6">
         <f t="shared" si="50"/>
         <v>0</v>
       </c>
@@ -9386,7 +9201,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="46" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -9401,7 +9216,7 @@
         <v>81</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F46" s="1">
         <v>91</v>
@@ -9414,7 +9229,7 @@
         <v>31.120686707020965</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J46" s="1">
         <v>20</v>
@@ -9524,11 +9339,11 @@
         <f t="shared" si="46"/>
         <v>5.5645400733479775</v>
       </c>
-      <c r="AQ46" s="8">
+      <c r="AQ46" s="6">
         <f t="shared" si="49"/>
         <v>0</v>
       </c>
-      <c r="AR46" s="8">
+      <c r="AR46" s="6">
         <f t="shared" si="50"/>
         <v>0</v>
       </c>
@@ -9580,7 +9395,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="47" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -9595,7 +9410,7 @@
         <v>66</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F47" s="1">
         <v>79</v>
@@ -9608,7 +9423,7 @@
         <v>29.017447199265384</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J47" s="1">
         <v>30</v>
@@ -9718,11 +9533,11 @@
         <f t="shared" si="46"/>
         <v>5.1875043152146363</v>
       </c>
-      <c r="AQ47" s="8">
+      <c r="AQ47" s="6">
         <f t="shared" si="49"/>
         <v>0</v>
       </c>
-      <c r="AR47" s="8">
+      <c r="AR47" s="6">
         <f t="shared" si="50"/>
         <v>0</v>
       </c>
@@ -9774,7 +9589,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="48" spans="1:59" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -9789,7 +9604,7 @@
         <v>66</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F48" s="1">
         <v>96</v>
@@ -9802,7 +9617,7 @@
         <v>30.299204645878042</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="J48" s="1">
         <v>50</v>
@@ -9912,11 +9727,11 @@
         <f t="shared" si="46"/>
         <v>5.418021194399838</v>
       </c>
-      <c r="AQ48" s="8">
+      <c r="AQ48" s="6">
         <f t="shared" si="49"/>
         <v>0</v>
       </c>
-      <c r="AR48" s="8">
+      <c r="AR48" s="6">
         <f t="shared" si="50"/>
         <v>0</v>
       </c>
@@ -9970,26 +9785,26 @@
     </row>
   </sheetData>
   <dataValidations count="7">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"F,M"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"NF,ExF,F"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"0,lobectomie,pneumonectomie"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:P1048576 K2:L1048576 BN18:BN1048576 BH2:BL16 BH18:BL1048576 BN2:BN16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:P1048576 K2:L1048576 BN18:BN1048576 BH2:BL16 BH18:BL1048576 BN2:BN16" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"0,1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BG18:BG1048576 BG2:BG16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BG18:BG1048576 BG2:BG16" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"FPI,PHS,connectivite,inclassable,autre"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q1048576 BR2:BR1048576">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q1048576 BR2:BR1048576" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>0</formula1>
       <formula2>4</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R1048576 BT2:BT1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R1048576 BT2:BT1048576" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"0,1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>